<commit_message>
Update IESO report from GitHub Actions
</commit_message>
<xml_diff>
--- a/output/latest.xlsx
+++ b/output/latest.xlsx
@@ -493,7 +493,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>CreatedAt: 2026-03-04T22:20:16</t>
+          <t>CreatedAt: 2026-03-04T23:21:24</t>
         </is>
       </c>
       <c r="B1" s="3" t="n"/>
@@ -650,76 +650,76 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>46.8</v>
+        <v>44.72</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>35.33</v>
+        <v>40.62</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>35.02</v>
+        <v>35.29</v>
       </c>
       <c r="F4" s="3" t="n">
+        <v>35.54</v>
+      </c>
+      <c r="G4" s="3" t="n">
         <v>35.4</v>
       </c>
-      <c r="G4" s="3" t="n">
-        <v>35.68</v>
-      </c>
       <c r="H4" s="3" t="n">
-        <v>35.33</v>
+        <v>35.1</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>48.25</v>
+        <v>40.14</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>42.04</v>
+        <v>47</v>
       </c>
       <c r="K4" s="3" t="n">
+        <v>41.79</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>36.67</v>
+      </c>
+      <c r="M4" s="3" t="n">
         <v>37.12</v>
       </c>
-      <c r="L4" s="3" t="n">
-        <v>35.67</v>
-      </c>
-      <c r="M4" s="3" t="n">
-        <v>35.05</v>
-      </c>
       <c r="N4" s="3" t="n">
-        <v>40.33</v>
+        <v>37.24</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>36.89</v>
+        <v>35.36</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>40.1</v>
+        <v>37.19</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>37.19</v>
+        <v>37.15</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>40.13</v>
+        <v>36.93</v>
       </c>
       <c r="S4" s="3" t="n">
-        <v>55.05</v>
+        <v>51.67</v>
       </c>
       <c r="T4" s="3" t="n">
-        <v>50.73</v>
+        <v>50.54</v>
       </c>
       <c r="U4" s="3" t="n">
-        <v>45.16</v>
+        <v>50.63</v>
       </c>
       <c r="V4" s="3" t="n">
-        <v>60.42</v>
+        <v>63.25</v>
       </c>
       <c r="W4" s="3" t="n">
-        <v>65.38</v>
+        <v>64.56</v>
       </c>
       <c r="X4" s="3" t="n">
-        <v>54.16</v>
+        <v>55.22</v>
       </c>
       <c r="Y4" s="3" t="n">
-        <v>50.9</v>
+        <v>48.75</v>
       </c>
       <c r="Z4" s="3" t="n">
-        <v>40.49</v>
+        <v>40.57</v>
       </c>
     </row>
     <row r="5">
@@ -818,16 +818,16 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>-0.35</v>
+        <v>0.04</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>-0.35</v>
+        <v>-0.39</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-0.14</v>
+        <v>-0.11</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>-0.14</v>
@@ -836,58 +836,58 @@
         <v>-0.25</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>-0.53</v>
+        <v>-0.36</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>-0.71</v>
+        <v>-0.8</v>
       </c>
       <c r="K6" s="3" t="n">
+        <v>-0.75</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>-0.62</v>
+      </c>
+      <c r="M6" s="3" t="n">
         <v>-0.59</v>
-      </c>
-      <c r="L6" s="3" t="n">
-        <v>-0.57</v>
-      </c>
-      <c r="M6" s="3" t="n">
-        <v>-0.63</v>
       </c>
       <c r="N6" s="3" t="n">
         <v>-0.5600000000000001</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>-0.44</v>
+        <v>-0.5</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>-0.52</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>-0.52</v>
+        <v>-0.59</v>
       </c>
       <c r="R6" s="3" t="n">
-        <v>-0.6</v>
+        <v>-0.7</v>
       </c>
       <c r="S6" s="3" t="n">
-        <v>-1.49</v>
+        <v>-1.5</v>
       </c>
       <c r="T6" s="3" t="n">
-        <v>-1.62</v>
+        <v>-1.72</v>
       </c>
       <c r="U6" s="3" t="n">
-        <v>-1.67</v>
+        <v>-1.82</v>
       </c>
       <c r="V6" s="3" t="n">
-        <v>-2.42</v>
+        <v>-2.59</v>
       </c>
       <c r="W6" s="3" t="n">
-        <v>-2.62</v>
+        <v>-2.52</v>
       </c>
       <c r="X6" s="3" t="n">
-        <v>-1.57</v>
+        <v>-1.6</v>
       </c>
       <c r="Y6" s="3" t="n">
-        <v>-0.97</v>
+        <v>-0.78</v>
       </c>
       <c r="Z6" s="3" t="n">
-        <v>-0.36</v>
+        <v>-0.37</v>
       </c>
     </row>
     <row r="7">
@@ -1070,76 +1070,76 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>48.4</v>
+        <v>46.25</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>36.6</v>
+        <v>41.79</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>36.32</v>
+        <v>36.67</v>
       </c>
       <c r="F9" s="3" t="n">
+        <v>36.98</v>
+      </c>
+      <c r="G9" s="3" t="n">
         <v>36.83</v>
       </c>
-      <c r="G9" s="3" t="n">
-        <v>37.12</v>
-      </c>
       <c r="H9" s="3" t="n">
-        <v>36.49</v>
+        <v>36.17</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>49.52</v>
+        <v>41.12</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>42.42</v>
+        <v>47.32</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>37.86</v>
+        <v>42.59</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>36.68</v>
+        <v>37.71</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>35.86</v>
+        <v>38.09</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>41.47</v>
+        <v>38.33</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>38.13</v>
+        <v>36.55</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>41.24</v>
+        <v>38.29</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>38.29</v>
+        <v>38.25</v>
       </c>
       <c r="R9" s="3" t="n">
-        <v>41.57</v>
+        <v>38.24</v>
       </c>
       <c r="S9" s="3" t="n">
-        <v>56.65</v>
+        <v>53.16</v>
       </c>
       <c r="T9" s="3" t="n">
-        <v>50.73</v>
+        <v>50.54</v>
       </c>
       <c r="U9" s="3" t="n">
-        <v>45.74</v>
+        <v>51.23</v>
       </c>
       <c r="V9" s="3" t="n">
-        <v>60.83</v>
+        <v>63.68</v>
       </c>
       <c r="W9" s="3" t="n">
-        <v>67.45</v>
+        <v>66.48</v>
       </c>
       <c r="X9" s="3" t="n">
-        <v>55.84</v>
+        <v>56.88</v>
       </c>
       <c r="Y9" s="3" t="n">
-        <v>52.49</v>
+        <v>50.24</v>
       </c>
       <c r="Z9" s="3" t="n">
-        <v>41.9</v>
+        <v>41.94</v>
       </c>
     </row>
     <row r="10">
@@ -1238,76 +1238,76 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>1.6</v>
+        <v>1.62</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0.91</v>
+        <v>1.21</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.99</v>
       </c>
       <c r="F11" s="3" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="G11" s="3" t="n">
         <v>1.29</v>
       </c>
-      <c r="G11" s="3" t="n">
-        <v>1.3</v>
-      </c>
       <c r="H11" s="3" t="n">
-        <v>0.91</v>
+        <v>0.83</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0.74</v>
+        <v>0.62</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>-0.34</v>
+        <v>-0.47</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0.15</v>
+        <v>0.04</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>0.44</v>
+        <v>0.41</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0.18</v>
+        <v>0.38</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>0.58</v>
+        <v>0.54</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>0.8</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>0.62</v>
+        <v>0.54</v>
       </c>
       <c r="Q11" s="3" t="n">
-        <v>0.57</v>
+        <v>0.5</v>
       </c>
       <c r="R11" s="3" t="n">
-        <v>0.83</v>
+        <v>0.61</v>
       </c>
       <c r="S11" s="3" t="n">
-        <v>0.11</v>
+        <v>0</v>
       </c>
       <c r="T11" s="3" t="n">
-        <v>-1.62</v>
+        <v>-1.72</v>
       </c>
       <c r="U11" s="3" t="n">
-        <v>-1.1</v>
+        <v>-1.23</v>
       </c>
       <c r="V11" s="3" t="n">
-        <v>-2.01</v>
+        <v>-2.17</v>
       </c>
       <c r="W11" s="3" t="n">
-        <v>-0.54</v>
+        <v>-0.6</v>
       </c>
       <c r="X11" s="3" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="Y11" s="3" t="n">
-        <v>0.63</v>
+        <v>0.7</v>
       </c>
       <c r="Z11" s="3" t="n">
-        <v>1.05</v>
+        <v>1.01</v>
       </c>
     </row>
     <row r="12">
@@ -1490,76 +1490,76 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>48.4</v>
+        <v>46.25</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>36.64</v>
+        <v>41.79</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>36.36</v>
+        <v>36.67</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>36.83</v>
+        <v>37.02</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>37.16</v>
+        <v>36.87</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>36.49</v>
+        <v>36.21</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>49.52</v>
+        <v>41.12</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>42.42</v>
+        <v>47.32</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>37.86</v>
+        <v>42.63</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>36.68</v>
+        <v>37.71</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>35.86</v>
+        <v>38.13</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>41.51</v>
+        <v>38.37</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>38.13</v>
+        <v>36.55</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>41.28</v>
+        <v>38.29</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>38.29</v>
+        <v>38.25</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>41.57</v>
+        <v>38.24</v>
       </c>
       <c r="S14" s="3" t="n">
-        <v>56.71</v>
+        <v>140.9</v>
       </c>
       <c r="T14" s="3" t="n">
-        <v>50.73</v>
+        <v>50.54</v>
       </c>
       <c r="U14" s="3" t="n">
-        <v>45.74</v>
+        <v>51.23</v>
       </c>
       <c r="V14" s="3" t="n">
-        <v>60.89</v>
+        <v>63.68</v>
       </c>
       <c r="W14" s="3" t="n">
-        <v>67.45</v>
+        <v>66.48</v>
       </c>
       <c r="X14" s="3" t="n">
-        <v>55.9</v>
+        <v>56.94</v>
       </c>
       <c r="Y14" s="3" t="n">
-        <v>52.55</v>
+        <v>50.24</v>
       </c>
       <c r="Z14" s="3" t="n">
-        <v>41.9</v>
+        <v>41.94</v>
       </c>
     </row>
     <row r="15">
@@ -1622,7 +1622,7 @@
         <v>0</v>
       </c>
       <c r="S15" s="3" t="n">
-        <v>0</v>
+        <v>87.73</v>
       </c>
       <c r="T15" s="3" t="n">
         <v>0</v>
@@ -1658,76 +1658,76 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>1.6</v>
+        <v>1.62</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0.95</v>
+        <v>1.21</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>1.29</v>
+        <v>1.37</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>1.34</v>
+        <v>1.33</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0.91</v>
+        <v>0.87</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>0.74</v>
+        <v>0.62</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>-0.34</v>
+        <v>-0.47</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>0.15</v>
+        <v>0.09</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>0.44</v>
+        <v>0.41</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0.18</v>
+        <v>0.42</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>0.62</v>
+        <v>0.58</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>0.8</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>0.66</v>
+        <v>0.54</v>
       </c>
       <c r="Q16" s="3" t="n">
-        <v>0.57</v>
+        <v>0.5</v>
       </c>
       <c r="R16" s="3" t="n">
-        <v>0.83</v>
+        <v>0.61</v>
       </c>
       <c r="S16" s="3" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="T16" s="3" t="n">
-        <v>-1.62</v>
+        <v>-1.72</v>
       </c>
       <c r="U16" s="3" t="n">
-        <v>-1.1</v>
+        <v>-1.23</v>
       </c>
       <c r="V16" s="3" t="n">
-        <v>-1.95</v>
+        <v>-2.17</v>
       </c>
       <c r="W16" s="3" t="n">
-        <v>-0.54</v>
+        <v>-0.6</v>
       </c>
       <c r="X16" s="3" t="n">
-        <v>0.17</v>
+        <v>0.11</v>
       </c>
       <c r="Y16" s="3" t="n">
-        <v>0.68</v>
+        <v>0.7</v>
       </c>
       <c r="Z16" s="3" t="n">
-        <v>1.05</v>
+        <v>1.01</v>
       </c>
     </row>
     <row r="17">
@@ -1910,76 +1910,76 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>46.52</v>
+        <v>44.5</v>
       </c>
       <c r="D19" s="3" t="n">
+        <v>40.38</v>
+      </c>
+      <c r="E19" s="3" t="n">
         <v>35.12</v>
       </c>
-      <c r="E19" s="3" t="n">
-        <v>34.85</v>
-      </c>
       <c r="F19" s="3" t="n">
+        <v>35.33</v>
+      </c>
+      <c r="G19" s="3" t="n">
         <v>35.22</v>
       </c>
-      <c r="G19" s="3" t="n">
-        <v>35.5</v>
-      </c>
       <c r="H19" s="3" t="n">
+        <v>34.92</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>39.94</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>46.77</v>
+      </c>
+      <c r="K19" s="3" t="n">
+        <v>41.55</v>
+      </c>
+      <c r="L19" s="3" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="M19" s="3" t="n">
+        <v>36.94</v>
+      </c>
+      <c r="N19" s="3" t="n">
+        <v>37.02</v>
+      </c>
+      <c r="O19" s="3" t="n">
         <v>35.19</v>
       </c>
-      <c r="I19" s="3" t="n">
-        <v>48.01</v>
-      </c>
-      <c r="J19" s="3" t="n">
-        <v>41.84</v>
-      </c>
-      <c r="K19" s="3" t="n">
-        <v>36.9</v>
-      </c>
-      <c r="L19" s="3" t="n">
-        <v>35.46</v>
-      </c>
-      <c r="M19" s="3" t="n">
-        <v>34.85</v>
-      </c>
-      <c r="N19" s="3" t="n">
-        <v>40.13</v>
-      </c>
-      <c r="O19" s="3" t="n">
-        <v>36.78</v>
-      </c>
       <c r="P19" s="3" t="n">
-        <v>39.94</v>
+        <v>37.01</v>
       </c>
       <c r="Q19" s="3" t="n">
-        <v>37.08</v>
+        <v>36.97</v>
       </c>
       <c r="R19" s="3" t="n">
-        <v>39.98</v>
+        <v>36.75</v>
       </c>
       <c r="S19" s="3" t="n">
-        <v>54.68</v>
+        <v>51.22</v>
       </c>
       <c r="T19" s="3" t="n">
-        <v>50.34</v>
+        <v>50.06</v>
       </c>
       <c r="U19" s="3" t="n">
-        <v>44.78</v>
+        <v>50.15</v>
       </c>
       <c r="V19" s="3" t="n">
-        <v>59.84</v>
+        <v>62.65</v>
       </c>
       <c r="W19" s="3" t="n">
-        <v>64.88</v>
+        <v>64.06999999999999</v>
       </c>
       <c r="X19" s="3" t="n">
-        <v>53.69</v>
+        <v>54.8</v>
       </c>
       <c r="Y19" s="3" t="n">
-        <v>50.55</v>
+        <v>48.42</v>
       </c>
       <c r="Z19" s="3" t="n">
-        <v>40.25</v>
+        <v>40.29</v>
       </c>
     </row>
     <row r="20">
@@ -2078,13 +2078,13 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>-0.28</v>
+        <v>-0.13</v>
       </c>
       <c r="D21" s="3" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="E21" s="3" t="n">
         <v>-0.5600000000000001</v>
-      </c>
-      <c r="E21" s="3" t="n">
-        <v>-0.52</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>-0.32</v>
@@ -2093,61 +2093,61 @@
         <v>-0.32</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>-0.39</v>
+        <v>-0.42</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>-0.77</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>-0.92</v>
+        <v>-1.03</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-1</v>
       </c>
       <c r="L21" s="3" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="M21" s="3" t="n">
         <v>-0.78</v>
       </c>
-      <c r="M21" s="3" t="n">
-        <v>-0.84</v>
-      </c>
       <c r="N21" s="3" t="n">
-        <v>-0.76</v>
+        <v>-0.78</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>-0.55</v>
+        <v>-0.67</v>
       </c>
       <c r="P21" s="3" t="n">
-        <v>-0.68</v>
+        <v>-0.74</v>
       </c>
       <c r="Q21" s="3" t="n">
-        <v>-0.63</v>
+        <v>-0.78</v>
       </c>
       <c r="R21" s="3" t="n">
-        <v>-0.76</v>
+        <v>-0.88</v>
       </c>
       <c r="S21" s="3" t="n">
-        <v>-1.86</v>
+        <v>-1.95</v>
       </c>
       <c r="T21" s="3" t="n">
-        <v>-2.01</v>
+        <v>-2.2</v>
       </c>
       <c r="U21" s="3" t="n">
-        <v>-2.06</v>
+        <v>-2.31</v>
       </c>
       <c r="V21" s="3" t="n">
-        <v>-2.99</v>
+        <v>-3.2</v>
       </c>
       <c r="W21" s="3" t="n">
-        <v>-3.11</v>
+        <v>-3.01</v>
       </c>
       <c r="X21" s="3" t="n">
-        <v>-2.04</v>
+        <v>-2.03</v>
       </c>
       <c r="Y21" s="3" t="n">
-        <v>-1.31</v>
+        <v>-1.11</v>
       </c>
       <c r="Z21" s="3" t="n">
-        <v>-0.6</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="22">
@@ -2330,76 +2330,76 @@
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>46.52</v>
+        <v>44.5</v>
       </c>
       <c r="D24" s="3" t="n">
+        <v>40.38</v>
+      </c>
+      <c r="E24" s="3" t="n">
         <v>35.12</v>
       </c>
-      <c r="E24" s="3" t="n">
-        <v>34.85</v>
-      </c>
       <c r="F24" s="3" t="n">
+        <v>35.33</v>
+      </c>
+      <c r="G24" s="3" t="n">
         <v>35.22</v>
       </c>
-      <c r="G24" s="3" t="n">
-        <v>35.5</v>
-      </c>
       <c r="H24" s="3" t="n">
+        <v>34.92</v>
+      </c>
+      <c r="I24" s="3" t="n">
+        <v>39.94</v>
+      </c>
+      <c r="J24" s="3" t="n">
+        <v>46.77</v>
+      </c>
+      <c r="K24" s="3" t="n">
+        <v>41.55</v>
+      </c>
+      <c r="L24" s="3" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="M24" s="3" t="n">
+        <v>36.94</v>
+      </c>
+      <c r="N24" s="3" t="n">
+        <v>37.02</v>
+      </c>
+      <c r="O24" s="3" t="n">
         <v>35.19</v>
       </c>
-      <c r="I24" s="3" t="n">
-        <v>48.01</v>
-      </c>
-      <c r="J24" s="3" t="n">
-        <v>41.84</v>
-      </c>
-      <c r="K24" s="3" t="n">
-        <v>36.9</v>
-      </c>
-      <c r="L24" s="3" t="n">
-        <v>35.46</v>
-      </c>
-      <c r="M24" s="3" t="n">
-        <v>34.85</v>
-      </c>
-      <c r="N24" s="3" t="n">
-        <v>40.13</v>
-      </c>
-      <c r="O24" s="3" t="n">
-        <v>36.78</v>
-      </c>
       <c r="P24" s="3" t="n">
-        <v>39.94</v>
+        <v>37.01</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>37.08</v>
+        <v>36.97</v>
       </c>
       <c r="R24" s="3" t="n">
-        <v>39.98</v>
+        <v>36.75</v>
       </c>
       <c r="S24" s="3" t="n">
-        <v>54.68</v>
+        <v>51.22</v>
       </c>
       <c r="T24" s="3" t="n">
-        <v>50.34</v>
+        <v>50.06</v>
       </c>
       <c r="U24" s="3" t="n">
-        <v>44.78</v>
+        <v>50.15</v>
       </c>
       <c r="V24" s="3" t="n">
-        <v>59.84</v>
+        <v>62.65</v>
       </c>
       <c r="W24" s="3" t="n">
-        <v>64.88</v>
+        <v>64.06999999999999</v>
       </c>
       <c r="X24" s="3" t="n">
-        <v>53.69</v>
+        <v>54.8</v>
       </c>
       <c r="Y24" s="3" t="n">
-        <v>50.55</v>
+        <v>48.42</v>
       </c>
       <c r="Z24" s="3" t="n">
-        <v>40.25</v>
+        <v>40.29</v>
       </c>
     </row>
     <row r="25">
@@ -2498,13 +2498,13 @@
         </is>
       </c>
       <c r="C26" s="3" t="n">
-        <v>-0.28</v>
+        <v>-0.13</v>
       </c>
       <c r="D26" s="3" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="E26" s="3" t="n">
         <v>-0.5600000000000001</v>
-      </c>
-      <c r="E26" s="3" t="n">
-        <v>-0.52</v>
       </c>
       <c r="F26" s="3" t="n">
         <v>-0.32</v>
@@ -2513,61 +2513,61 @@
         <v>-0.32</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>-0.39</v>
+        <v>-0.42</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>-0.77</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>-0.92</v>
+        <v>-1.03</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-1</v>
       </c>
       <c r="L26" s="3" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="M26" s="3" t="n">
         <v>-0.78</v>
       </c>
-      <c r="M26" s="3" t="n">
-        <v>-0.84</v>
-      </c>
       <c r="N26" s="3" t="n">
-        <v>-0.76</v>
+        <v>-0.78</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>-0.55</v>
+        <v>-0.67</v>
       </c>
       <c r="P26" s="3" t="n">
-        <v>-0.68</v>
+        <v>-0.74</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>-0.63</v>
+        <v>-0.78</v>
       </c>
       <c r="R26" s="3" t="n">
-        <v>-0.76</v>
+        <v>-0.88</v>
       </c>
       <c r="S26" s="3" t="n">
-        <v>-1.86</v>
+        <v>-1.95</v>
       </c>
       <c r="T26" s="3" t="n">
-        <v>-2.01</v>
+        <v>-2.2</v>
       </c>
       <c r="U26" s="3" t="n">
-        <v>-2.06</v>
+        <v>-2.31</v>
       </c>
       <c r="V26" s="3" t="n">
-        <v>-2.99</v>
+        <v>-3.2</v>
       </c>
       <c r="W26" s="3" t="n">
-        <v>-3.11</v>
+        <v>-3.01</v>
       </c>
       <c r="X26" s="3" t="n">
-        <v>-2.04</v>
+        <v>-2.03</v>
       </c>
       <c r="Y26" s="3" t="n">
-        <v>-1.31</v>
+        <v>-1.11</v>
       </c>
       <c r="Z26" s="3" t="n">
-        <v>-0.6</v>
+        <v>-0.64</v>
       </c>
     </row>
     <row r="27">
@@ -2750,76 +2750,76 @@
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>46.07</v>
+        <v>44.01</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>34.78</v>
+        <v>39.9</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>34.58</v>
+        <v>34.85</v>
       </c>
       <c r="F29" s="3" t="n">
+        <v>35.02</v>
+      </c>
+      <c r="G29" s="3" t="n">
         <v>34.91</v>
       </c>
-      <c r="G29" s="3" t="n">
-        <v>35.22</v>
-      </c>
       <c r="H29" s="3" t="n">
-        <v>34.91</v>
+        <v>34.61</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>47.64</v>
+        <v>39.67</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>41.51</v>
+        <v>46.45</v>
       </c>
       <c r="K29" s="3" t="n">
+        <v>41.19</v>
+      </c>
+      <c r="L29" s="3" t="n">
+        <v>36.14</v>
+      </c>
+      <c r="M29" s="3" t="n">
         <v>36.61</v>
       </c>
-      <c r="L29" s="3" t="n">
-        <v>35.15</v>
-      </c>
-      <c r="M29" s="3" t="n">
-        <v>34.48</v>
-      </c>
       <c r="N29" s="3" t="n">
-        <v>39.78</v>
+        <v>36.62</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>36.49</v>
+        <v>34.81</v>
       </c>
       <c r="P29" s="3" t="n">
-        <v>39.67</v>
+        <v>36.65</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>36.83</v>
+        <v>36.65</v>
       </c>
       <c r="R29" s="3" t="n">
-        <v>39.7</v>
+        <v>36.39</v>
       </c>
       <c r="S29" s="3" t="n">
-        <v>54.11</v>
+        <v>50.54</v>
       </c>
       <c r="T29" s="3" t="n">
-        <v>49.86</v>
+        <v>49.54</v>
       </c>
       <c r="U29" s="3" t="n">
-        <v>44.31</v>
+        <v>49.58</v>
       </c>
       <c r="V29" s="3" t="n">
-        <v>59.11</v>
+        <v>61.94</v>
       </c>
       <c r="W29" s="3" t="n">
-        <v>64.14</v>
+        <v>63.28</v>
       </c>
       <c r="X29" s="3" t="n">
-        <v>53.07</v>
+        <v>54.12</v>
       </c>
       <c r="Y29" s="3" t="n">
-        <v>49.96</v>
+        <v>47.86</v>
       </c>
       <c r="Z29" s="3" t="n">
-        <v>39.82</v>
+        <v>39.85</v>
       </c>
     </row>
     <row r="30">
@@ -2918,76 +2918,76 @@
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>-0.74</v>
+        <v>-0.62</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>-0.9</v>
+        <v>-0.68</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>-0.8</v>
+        <v>-0.84</v>
       </c>
       <c r="F31" s="3" t="n">
         <v>-0.63</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>-0.6</v>
+        <v>-0.63</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>-0.66</v>
+        <v>-0.73</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>-1.14</v>
+        <v>-0.83</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>-1.25</v>
+        <v>-1.35</v>
       </c>
       <c r="K31" s="3" t="n">
+        <v>-1.36</v>
+      </c>
+      <c r="L31" s="3" t="n">
+        <v>-1.16</v>
+      </c>
+      <c r="M31" s="3" t="n">
         <v>-1.1</v>
       </c>
-      <c r="L31" s="3" t="n">
-        <v>-1.09</v>
-      </c>
-      <c r="M31" s="3" t="n">
-        <v>-1.21</v>
-      </c>
       <c r="N31" s="3" t="n">
-        <v>-1.11</v>
+        <v>-1.17</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>-0.84</v>
+        <v>-1.04</v>
       </c>
       <c r="P31" s="3" t="n">
-        <v>-0.95</v>
+        <v>-1.1</v>
       </c>
       <c r="Q31" s="3" t="n">
-        <v>-0.88</v>
+        <v>-1.1</v>
       </c>
       <c r="R31" s="3" t="n">
-        <v>-1.03</v>
+        <v>-1.24</v>
       </c>
       <c r="S31" s="3" t="n">
-        <v>-2.43</v>
+        <v>-2.63</v>
       </c>
       <c r="T31" s="3" t="n">
-        <v>-2.49</v>
+        <v>-2.72</v>
       </c>
       <c r="U31" s="3" t="n">
-        <v>-2.53</v>
+        <v>-2.88</v>
       </c>
       <c r="V31" s="3" t="n">
-        <v>-3.72</v>
+        <v>-3.9</v>
       </c>
       <c r="W31" s="3" t="n">
-        <v>-3.85</v>
+        <v>-3.8</v>
       </c>
       <c r="X31" s="3" t="n">
-        <v>-2.65</v>
+        <v>-2.71</v>
       </c>
       <c r="Y31" s="3" t="n">
-        <v>-1.9</v>
+        <v>-1.68</v>
       </c>
       <c r="Z31" s="3" t="n">
-        <v>-1.04</v>
+        <v>-1.08</v>
       </c>
     </row>
     <row r="32">
@@ -3170,76 +3170,76 @@
         </is>
       </c>
       <c r="C34" s="3" t="n">
-        <v>49.11</v>
+        <v>46.98</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>36.94</v>
+        <v>42.23</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>36.62</v>
+        <v>37.02</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>37.22</v>
+        <v>37.44</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>37.55</v>
+        <v>37.29</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>36.79</v>
+        <v>36.43</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>49.62</v>
+        <v>41.16</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>42.8</v>
+        <v>47.7</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>37.79</v>
+        <v>42.55</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>36.79</v>
+        <v>37.87</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>35.83</v>
+        <v>38.09</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>41.68</v>
+        <v>38.61</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>38.37</v>
+        <v>36.89</v>
       </c>
       <c r="P34" s="3" t="n">
-        <v>41.32</v>
+        <v>38.44</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>38.36</v>
+        <v>38.4</v>
       </c>
       <c r="R34" s="3" t="n">
-        <v>41.91</v>
+        <v>38.63</v>
       </c>
       <c r="S34" s="3" t="n">
-        <v>57</v>
+        <v>77.23</v>
       </c>
       <c r="T34" s="3" t="n">
-        <v>50.88</v>
+        <v>50.79</v>
       </c>
       <c r="U34" s="3" t="n">
-        <v>45.74</v>
+        <v>51.28</v>
       </c>
       <c r="V34" s="3" t="n">
-        <v>61.48</v>
+        <v>64.36</v>
       </c>
       <c r="W34" s="3" t="n">
-        <v>68.75</v>
+        <v>67.69</v>
       </c>
       <c r="X34" s="3" t="n">
-        <v>56.29</v>
+        <v>57.28</v>
       </c>
       <c r="Y34" s="3" t="n">
-        <v>53.08</v>
+        <v>50.54</v>
       </c>
       <c r="Z34" s="3" t="n">
-        <v>42.2</v>
+        <v>42.24</v>
       </c>
     </row>
     <row r="35">
@@ -3302,7 +3302,7 @@
         <v>0</v>
       </c>
       <c r="S35" s="3" t="n">
-        <v>0</v>
+        <v>23.69</v>
       </c>
       <c r="T35" s="3" t="n">
         <v>0</v>
@@ -3338,76 +3338,76 @@
         </is>
       </c>
       <c r="C36" s="3" t="n">
-        <v>2.31</v>
+        <v>2.35</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>1.26</v>
+        <v>1.65</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>1.25</v>
+        <v>1.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>1.73</v>
+        <v>1.75</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>1.21</v>
+        <v>1.09</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>0.84</v>
+        <v>0.66</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>0.04</v>
+        <v>-0.1</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>0.55</v>
+        <v>0.57</v>
       </c>
       <c r="M36" s="3" t="n">
-        <v>0.14</v>
+        <v>0.38</v>
       </c>
       <c r="N36" s="3" t="n">
-        <v>0.79</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="O36" s="3" t="n">
-        <v>1.04</v>
+        <v>1.03</v>
       </c>
       <c r="P36" s="3" t="n">
-        <v>0.7</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Q36" s="3" t="n">
         <v>0.65</v>
       </c>
       <c r="R36" s="3" t="n">
-        <v>1.17</v>
+        <v>1</v>
       </c>
       <c r="S36" s="3" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="T36" s="3" t="n">
+        <v>-1.47</v>
+      </c>
+      <c r="U36" s="3" t="n">
+        <v>-1.18</v>
+      </c>
+      <c r="V36" s="3" t="n">
+        <v>-1.48</v>
+      </c>
+      <c r="W36" s="3" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="X36" s="3" t="n">
         <v>0.46</v>
       </c>
-      <c r="T36" s="3" t="n">
-        <v>-1.48</v>
-      </c>
-      <c r="U36" s="3" t="n">
-        <v>-1.1</v>
-      </c>
-      <c r="V36" s="3" t="n">
-        <v>-1.35</v>
-      </c>
-      <c r="W36" s="3" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="X36" s="3" t="n">
-        <v>0.5600000000000001</v>
-      </c>
       <c r="Y36" s="3" t="n">
-        <v>1.22</v>
+        <v>1.01</v>
       </c>
       <c r="Z36" s="3" t="n">
-        <v>1.35</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="37">
@@ -3590,76 +3590,76 @@
         </is>
       </c>
       <c r="C39" s="3" t="n">
-        <v>46.8</v>
+        <v>44.72</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>35.33</v>
+        <v>40.62</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>35.02</v>
+        <v>35.29</v>
       </c>
       <c r="F39" s="3" t="n">
+        <v>35.54</v>
+      </c>
+      <c r="G39" s="3" t="n">
         <v>35.4</v>
       </c>
-      <c r="G39" s="3" t="n">
-        <v>35.68</v>
-      </c>
       <c r="H39" s="3" t="n">
-        <v>35.33</v>
+        <v>35.1</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>48.25</v>
+        <v>40.14</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>42.04</v>
+        <v>47</v>
       </c>
       <c r="K39" s="3" t="n">
+        <v>41.79</v>
+      </c>
+      <c r="L39" s="3" t="n">
+        <v>36.67</v>
+      </c>
+      <c r="M39" s="3" t="n">
         <v>37.12</v>
       </c>
-      <c r="L39" s="3" t="n">
-        <v>35.67</v>
-      </c>
-      <c r="M39" s="3" t="n">
-        <v>35.05</v>
-      </c>
       <c r="N39" s="3" t="n">
-        <v>40.33</v>
+        <v>37.24</v>
       </c>
       <c r="O39" s="3" t="n">
-        <v>36.89</v>
+        <v>35.36</v>
       </c>
       <c r="P39" s="3" t="n">
-        <v>40.1</v>
+        <v>37.19</v>
       </c>
       <c r="Q39" s="3" t="n">
-        <v>37.19</v>
+        <v>37.15</v>
       </c>
       <c r="R39" s="3" t="n">
-        <v>40.13</v>
+        <v>36.93</v>
       </c>
       <c r="S39" s="3" t="n">
-        <v>55.05</v>
+        <v>51.67</v>
       </c>
       <c r="T39" s="3" t="n">
-        <v>50.73</v>
+        <v>50.54</v>
       </c>
       <c r="U39" s="3" t="n">
-        <v>45.16</v>
+        <v>50.63</v>
       </c>
       <c r="V39" s="3" t="n">
-        <v>60.42</v>
+        <v>63.25</v>
       </c>
       <c r="W39" s="3" t="n">
-        <v>65.38</v>
+        <v>64.56</v>
       </c>
       <c r="X39" s="3" t="n">
-        <v>54.16</v>
+        <v>55.22</v>
       </c>
       <c r="Y39" s="3" t="n">
-        <v>50.9</v>
+        <v>48.75</v>
       </c>
       <c r="Z39" s="3" t="n">
-        <v>40.49</v>
+        <v>40.57</v>
       </c>
     </row>
     <row r="40">
@@ -3758,16 +3758,16 @@
         </is>
       </c>
       <c r="C41" s="3" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>-0.35</v>
+        <v>0.04</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>-0.35</v>
+        <v>-0.39</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>-0.14</v>
+        <v>-0.11</v>
       </c>
       <c r="G41" s="3" t="n">
         <v>-0.14</v>
@@ -3776,58 +3776,58 @@
         <v>-0.25</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>-0.53</v>
+        <v>-0.36</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>-0.71</v>
+        <v>-0.8</v>
       </c>
       <c r="K41" s="3" t="n">
+        <v>-0.75</v>
+      </c>
+      <c r="L41" s="3" t="n">
+        <v>-0.62</v>
+      </c>
+      <c r="M41" s="3" t="n">
         <v>-0.59</v>
-      </c>
-      <c r="L41" s="3" t="n">
-        <v>-0.57</v>
-      </c>
-      <c r="M41" s="3" t="n">
-        <v>-0.63</v>
       </c>
       <c r="N41" s="3" t="n">
         <v>-0.5600000000000001</v>
       </c>
       <c r="O41" s="3" t="n">
-        <v>-0.44</v>
+        <v>-0.5</v>
       </c>
       <c r="P41" s="3" t="n">
-        <v>-0.52</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="Q41" s="3" t="n">
-        <v>-0.52</v>
+        <v>-0.59</v>
       </c>
       <c r="R41" s="3" t="n">
-        <v>-0.6</v>
+        <v>-0.7</v>
       </c>
       <c r="S41" s="3" t="n">
-        <v>-1.49</v>
+        <v>-1.5</v>
       </c>
       <c r="T41" s="3" t="n">
-        <v>-1.62</v>
+        <v>-1.72</v>
       </c>
       <c r="U41" s="3" t="n">
-        <v>-1.67</v>
+        <v>-1.82</v>
       </c>
       <c r="V41" s="3" t="n">
-        <v>-2.42</v>
+        <v>-2.59</v>
       </c>
       <c r="W41" s="3" t="n">
-        <v>-2.62</v>
+        <v>-2.52</v>
       </c>
       <c r="X41" s="3" t="n">
-        <v>-1.57</v>
+        <v>-1.6</v>
       </c>
       <c r="Y41" s="3" t="n">
-        <v>-0.97</v>
+        <v>-0.78</v>
       </c>
       <c r="Z41" s="3" t="n">
-        <v>-0.36</v>
+        <v>-0.37</v>
       </c>
     </row>
     <row r="42">
@@ -4010,76 +4010,76 @@
         </is>
       </c>
       <c r="C44" s="3" t="n">
-        <v>48</v>
+        <v>45.77</v>
       </c>
       <c r="D44" s="3" t="n">
+        <v>41.66</v>
+      </c>
+      <c r="E44" s="3" t="n">
         <v>36.56</v>
       </c>
-      <c r="E44" s="3" t="n">
-        <v>36.24</v>
-      </c>
       <c r="F44" s="3" t="n">
-        <v>36.49</v>
+        <v>36.6</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>36.74</v>
+        <v>36.42</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>36.42</v>
+        <v>36.17</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>50.03</v>
+        <v>41.58</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>43.67</v>
+        <v>48.77</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>38.25</v>
+        <v>43.15</v>
       </c>
       <c r="L44" s="3" t="n">
-        <v>36.6</v>
+        <v>37.67</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>35.97</v>
+        <v>38.05</v>
       </c>
       <c r="N44" s="3" t="n">
-        <v>41.35</v>
+        <v>38.22</v>
       </c>
       <c r="O44" s="3" t="n">
-        <v>37.71</v>
+        <v>36.18</v>
       </c>
       <c r="P44" s="3" t="n">
-        <v>41.07</v>
+        <v>38.17</v>
       </c>
       <c r="Q44" s="3" t="n">
         <v>38.13</v>
       </c>
       <c r="R44" s="3" t="n">
-        <v>41.27</v>
+        <v>38.09</v>
       </c>
       <c r="S44" s="3" t="n">
-        <v>57.75</v>
+        <v>54.3</v>
       </c>
       <c r="T44" s="3" t="n">
-        <v>53.53</v>
+        <v>53.44</v>
       </c>
       <c r="U44" s="3" t="n">
-        <v>47.84</v>
+        <v>53.58</v>
       </c>
       <c r="V44" s="3" t="n">
-        <v>64.05</v>
+        <v>67.05</v>
       </c>
       <c r="W44" s="3" t="n">
-        <v>69.31</v>
+        <v>68.38</v>
       </c>
       <c r="X44" s="3" t="n">
-        <v>56.87</v>
+        <v>57.99</v>
       </c>
       <c r="Y44" s="3" t="n">
-        <v>53.03</v>
+        <v>50.65</v>
       </c>
       <c r="Z44" s="3" t="n">
-        <v>42.03</v>
+        <v>42.11</v>
       </c>
     </row>
     <row r="45">
@@ -4178,73 +4178,73 @@
         </is>
       </c>
       <c r="C46" s="3" t="n">
-        <v>1.2</v>
+        <v>1.14</v>
       </c>
       <c r="D46" s="3" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="E46" s="3" t="n">
         <v>0.88</v>
-      </c>
-      <c r="E46" s="3" t="n">
-        <v>0.87</v>
       </c>
       <c r="F46" s="3" t="n">
         <v>0.95</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>0.92</v>
+        <v>0.87</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>0.84</v>
+        <v>0.83</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>1.25</v>
+        <v>1.08</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>0.54</v>
+        <v>0.6</v>
       </c>
       <c r="L46" s="3" t="n">
-        <v>0.37</v>
+        <v>0.38</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>0.29</v>
+        <v>0.34</v>
       </c>
       <c r="N46" s="3" t="n">
-        <v>0.45</v>
+        <v>0.42</v>
       </c>
       <c r="O46" s="3" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="P46" s="3" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="Q46" s="3" t="n">
         <v>0.38</v>
       </c>
-      <c r="P46" s="3" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="Q46" s="3" t="n">
-        <v>0.42</v>
-      </c>
       <c r="R46" s="3" t="n">
-        <v>0.54</v>
+        <v>0.46</v>
       </c>
       <c r="S46" s="3" t="n">
-        <v>1.21</v>
+        <v>1.14</v>
       </c>
       <c r="T46" s="3" t="n">
         <v>1.18</v>
       </c>
       <c r="U46" s="3" t="n">
-        <v>1</v>
+        <v>1.13</v>
       </c>
       <c r="V46" s="3" t="n">
-        <v>1.22</v>
+        <v>1.21</v>
       </c>
       <c r="W46" s="3" t="n">
-        <v>1.32</v>
+        <v>1.3</v>
       </c>
       <c r="X46" s="3" t="n">
-        <v>1.14</v>
+        <v>1.16</v>
       </c>
       <c r="Y46" s="3" t="n">
-        <v>1.17</v>
+        <v>1.11</v>
       </c>
       <c r="Z46" s="3" t="n">
         <v>1.18</v>
@@ -4430,76 +4430,76 @@
         </is>
       </c>
       <c r="C49" s="3" t="n">
-        <v>46.43</v>
+        <v>44.19</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>35.9</v>
+        <v>40.86</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>35.52</v>
+        <v>35.83</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>35.68</v>
+        <v>35.79</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>35.43</v>
+        <v>35.05</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>33.85</v>
+        <v>33.59</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>44.67</v>
+        <v>37.05</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>38.73</v>
+        <v>43.26</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>34.1</v>
+        <v>38.5</v>
       </c>
       <c r="L49" s="3" t="n">
-        <v>34.28</v>
+        <v>35.25</v>
       </c>
       <c r="M49" s="3" t="n">
-        <v>35.83</v>
+        <v>37.86</v>
       </c>
       <c r="N49" s="3" t="n">
-        <v>40.97</v>
+        <v>37.87</v>
       </c>
       <c r="O49" s="3" t="n">
-        <v>37.26</v>
+        <v>35.79</v>
       </c>
       <c r="P49" s="3" t="n">
-        <v>40.66</v>
+        <v>37.79</v>
       </c>
       <c r="Q49" s="3" t="n">
-        <v>37.75</v>
+        <v>37.79</v>
       </c>
       <c r="R49" s="3" t="n">
-        <v>40.94</v>
+        <v>37.82</v>
       </c>
       <c r="S49" s="3" t="n">
-        <v>54.63</v>
+        <v>51.42</v>
       </c>
       <c r="T49" s="3" t="n">
-        <v>47.68</v>
+        <v>47.64</v>
       </c>
       <c r="U49" s="3" t="n">
-        <v>42.81</v>
+        <v>47.9</v>
       </c>
       <c r="V49" s="3" t="n">
-        <v>57.49</v>
+        <v>60.13</v>
       </c>
       <c r="W49" s="3" t="n">
-        <v>65.19</v>
+        <v>64.31999999999999</v>
       </c>
       <c r="X49" s="3" t="n">
-        <v>53.84</v>
+        <v>54.9</v>
       </c>
       <c r="Y49" s="3" t="n">
-        <v>52.71</v>
+        <v>50.24</v>
       </c>
       <c r="Z49" s="3" t="n">
-        <v>41.43</v>
+        <v>41.51</v>
       </c>
     </row>
     <row r="50">
@@ -4598,10 +4598,10 @@
         </is>
       </c>
       <c r="C51" s="3" t="n">
-        <v>-0.37</v>
+        <v>-0.44</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>0.22</v>
+        <v>0.29</v>
       </c>
       <c r="E51" s="3" t="n">
         <v>0.14</v>
@@ -4610,25 +4610,25 @@
         <v>0.14</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>-0.39</v>
+        <v>-0.49</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>-1.73</v>
+        <v>-1.75</v>
       </c>
       <c r="I51" s="3" t="n">
-        <v>-4.11</v>
+        <v>-3.45</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>-4.03</v>
+        <v>-4.54</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>-3.61</v>
+        <v>-4.04</v>
       </c>
       <c r="L51" s="3" t="n">
-        <v>-1.95</v>
+        <v>-2.04</v>
       </c>
       <c r="M51" s="3" t="n">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="N51" s="3" t="n">
         <v>0.08</v>
@@ -4643,28 +4643,28 @@
         <v>0.04</v>
       </c>
       <c r="R51" s="3" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="S51" s="3" t="n">
-        <v>-1.91</v>
+        <v>-1.75</v>
       </c>
       <c r="T51" s="3" t="n">
-        <v>-4.67</v>
+        <v>-4.62</v>
       </c>
       <c r="U51" s="3" t="n">
-        <v>-4.02</v>
+        <v>-4.55</v>
       </c>
       <c r="V51" s="3" t="n">
-        <v>-5.35</v>
+        <v>-5.71</v>
       </c>
       <c r="W51" s="3" t="n">
-        <v>-2.8</v>
+        <v>-2.77</v>
       </c>
       <c r="X51" s="3" t="n">
-        <v>-1.88</v>
+        <v>-1.92</v>
       </c>
       <c r="Y51" s="3" t="n">
-        <v>0.84</v>
+        <v>0.7</v>
       </c>
       <c r="Z51" s="3" t="n">
         <v>0.58</v>
@@ -4850,76 +4850,76 @@
         </is>
       </c>
       <c r="C54" s="3" t="n">
-        <v>48.75</v>
+        <v>46.34</v>
       </c>
       <c r="D54" s="3" t="n">
-        <v>37.13</v>
+        <v>42.23</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>36.36</v>
+        <v>36.75</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>36.79</v>
+        <v>36.94</v>
       </c>
       <c r="G54" s="3" t="n">
-        <v>36.44</v>
+        <v>36.12</v>
       </c>
       <c r="H54" s="3" t="n">
-        <v>35.65</v>
+        <v>35.38</v>
       </c>
       <c r="I54" s="3" t="n">
-        <v>46.95</v>
+        <v>38.98</v>
       </c>
       <c r="J54" s="3" t="n">
-        <v>40.92</v>
+        <v>45.83</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>35.92</v>
+        <v>40.68</v>
       </c>
       <c r="L54" s="3" t="n">
-        <v>35.35</v>
+        <v>36.53</v>
       </c>
       <c r="M54" s="3" t="n">
-        <v>35.19</v>
+        <v>37.34</v>
       </c>
       <c r="N54" s="3" t="n">
-        <v>40.41</v>
+        <v>37.57</v>
       </c>
       <c r="O54" s="3" t="n">
-        <v>36.67</v>
+        <v>35.43</v>
       </c>
       <c r="P54" s="3" t="n">
-        <v>39.63</v>
+        <v>37.01</v>
       </c>
       <c r="Q54" s="3" t="n">
-        <v>36.83</v>
+        <v>37.05</v>
       </c>
       <c r="R54" s="3" t="n">
-        <v>39.7</v>
+        <v>36.86</v>
       </c>
       <c r="S54" s="3" t="n">
-        <v>55.32</v>
+        <v>52.07</v>
       </c>
       <c r="T54" s="3" t="n">
-        <v>51.23</v>
+        <v>51.24</v>
       </c>
       <c r="U54" s="3" t="n">
-        <v>44.52</v>
+        <v>49.82</v>
       </c>
       <c r="V54" s="3" t="n">
-        <v>62.21</v>
+        <v>65.13</v>
       </c>
       <c r="W54" s="3" t="n">
-        <v>67.58</v>
+        <v>66.61</v>
       </c>
       <c r="X54" s="3" t="n">
-        <v>55.51</v>
+        <v>56.6</v>
       </c>
       <c r="Y54" s="3" t="n">
-        <v>52.02</v>
+        <v>49.39</v>
       </c>
       <c r="Z54" s="3" t="n">
-        <v>40.77</v>
+        <v>40.81</v>
       </c>
     </row>
     <row r="55">
@@ -5018,76 +5018,76 @@
         </is>
       </c>
       <c r="C56" s="3" t="n">
-        <v>1.95</v>
+        <v>1.71</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>1.45</v>
+        <v>1.65</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>0.98</v>
+        <v>1.07</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>1.25</v>
+        <v>1.29</v>
       </c>
       <c r="G56" s="3" t="n">
-        <v>0.62</v>
+        <v>0.58</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.04</v>
       </c>
       <c r="I56" s="3" t="n">
-        <v>-1.83</v>
+        <v>-1.52</v>
       </c>
       <c r="J56" s="3" t="n">
-        <v>-1.84</v>
+        <v>-1.97</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>-1.8</v>
+        <v>-1.87</v>
       </c>
       <c r="L56" s="3" t="n">
-        <v>-0.88</v>
+        <v>-0.77</v>
       </c>
       <c r="M56" s="3" t="n">
-        <v>-0.49</v>
+        <v>-0.37</v>
       </c>
       <c r="N56" s="3" t="n">
-        <v>-0.48</v>
+        <v>-0.23</v>
       </c>
       <c r="O56" s="3" t="n">
-        <v>-0.66</v>
+        <v>-0.43</v>
       </c>
       <c r="P56" s="3" t="n">
-        <v>-0.99</v>
+        <v>-0.74</v>
       </c>
       <c r="Q56" s="3" t="n">
-        <v>-0.88</v>
+        <v>-0.7</v>
       </c>
       <c r="R56" s="3" t="n">
-        <v>-1.03</v>
+        <v>-0.77</v>
       </c>
       <c r="S56" s="3" t="n">
-        <v>-1.22</v>
+        <v>-1.09</v>
       </c>
       <c r="T56" s="3" t="n">
-        <v>-1.13</v>
+        <v>-1.02</v>
       </c>
       <c r="U56" s="3" t="n">
-        <v>-2.32</v>
+        <v>-2.64</v>
       </c>
       <c r="V56" s="3" t="n">
-        <v>-0.62</v>
+        <v>-0.72</v>
       </c>
       <c r="W56" s="3" t="n">
-        <v>-0.41</v>
+        <v>-0.47</v>
       </c>
       <c r="X56" s="3" t="n">
-        <v>-0.22</v>
+        <v>-0.23</v>
       </c>
       <c r="Y56" s="3" t="n">
-        <v>0.16</v>
+        <v>-0.15</v>
       </c>
       <c r="Z56" s="3" t="n">
-        <v>-0.08</v>
+        <v>-0.12</v>
       </c>
     </row>
     <row r="57">
@@ -5270,76 +5270,76 @@
         </is>
       </c>
       <c r="C59" s="3" t="n">
-        <v>49.37</v>
+        <v>47.08</v>
       </c>
       <c r="D59" s="3" t="n">
+        <v>42.85</v>
+      </c>
+      <c r="E59" s="3" t="n">
         <v>37.68</v>
       </c>
-      <c r="E59" s="3" t="n">
-        <v>37.35</v>
-      </c>
       <c r="F59" s="3" t="n">
-        <v>37.57</v>
+        <v>37.72</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>37.83</v>
+        <v>37.49</v>
       </c>
       <c r="H59" s="3" t="n">
-        <v>37.49</v>
+        <v>37.24</v>
       </c>
       <c r="I59" s="3" t="n">
-        <v>51.62</v>
+        <v>42.86</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>45.1</v>
+        <v>50.37</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>39.66</v>
+        <v>44.74</v>
       </c>
       <c r="L59" s="3" t="n">
-        <v>37.98</v>
+        <v>39.1</v>
       </c>
       <c r="M59" s="3" t="n">
-        <v>37.36</v>
+        <v>39.53</v>
       </c>
       <c r="N59" s="3" t="n">
-        <v>43</v>
+        <v>39.74</v>
       </c>
       <c r="O59" s="3" t="n">
-        <v>39.13</v>
+        <v>37.59</v>
       </c>
       <c r="P59" s="3" t="n">
-        <v>42.71</v>
+        <v>39.65</v>
       </c>
       <c r="Q59" s="3" t="n">
         <v>39.61</v>
       </c>
       <c r="R59" s="3" t="n">
-        <v>42.83</v>
+        <v>39.53</v>
       </c>
       <c r="S59" s="3" t="n">
-        <v>59.83</v>
+        <v>56.26</v>
       </c>
       <c r="T59" s="3" t="n">
-        <v>55.46</v>
+        <v>55.36</v>
       </c>
       <c r="U59" s="3" t="n">
-        <v>49.56</v>
+        <v>55.51</v>
       </c>
       <c r="V59" s="3" t="n">
-        <v>66.34999999999999</v>
+        <v>69.45999999999999</v>
       </c>
       <c r="W59" s="3" t="n">
-        <v>71.87</v>
+        <v>70.91</v>
       </c>
       <c r="X59" s="3" t="n">
-        <v>58.85</v>
+        <v>60.01</v>
       </c>
       <c r="Y59" s="3" t="n">
-        <v>54.77</v>
+        <v>52.25</v>
       </c>
       <c r="Z59" s="3" t="n">
-        <v>43.32</v>
+        <v>43.4</v>
       </c>
     </row>
     <row r="60">
@@ -5438,73 +5438,73 @@
         </is>
       </c>
       <c r="C61" s="3" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F61" s="3" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="G61" s="3" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="H61" s="3" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="I61" s="3" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="J61" s="3" t="n">
         <v>2.57</v>
       </c>
-      <c r="D61" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E61" s="3" t="n">
-        <v>1.98</v>
-      </c>
-      <c r="F61" s="3" t="n">
-        <v>2.03</v>
-      </c>
-      <c r="G61" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H61" s="3" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="I61" s="3" t="n">
-        <v>2.84</v>
-      </c>
-      <c r="J61" s="3" t="n">
-        <v>2.35</v>
-      </c>
       <c r="K61" s="3" t="n">
-        <v>1.94</v>
+        <v>2.19</v>
       </c>
       <c r="L61" s="3" t="n">
-        <v>1.75</v>
+        <v>1.8</v>
       </c>
       <c r="M61" s="3" t="n">
-        <v>1.68</v>
+        <v>1.82</v>
       </c>
       <c r="N61" s="3" t="n">
-        <v>2.11</v>
+        <v>1.95</v>
       </c>
       <c r="O61" s="3" t="n">
-        <v>1.8</v>
+        <v>1.73</v>
       </c>
       <c r="P61" s="3" t="n">
-        <v>2.09</v>
+        <v>1.9</v>
       </c>
       <c r="Q61" s="3" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="R61" s="3" t="n">
         <v>1.9</v>
       </c>
-      <c r="R61" s="3" t="n">
-        <v>2.1</v>
-      </c>
       <c r="S61" s="3" t="n">
-        <v>3.29</v>
+        <v>3.09</v>
       </c>
       <c r="T61" s="3" t="n">
-        <v>3.11</v>
+        <v>3.1</v>
       </c>
       <c r="U61" s="3" t="n">
-        <v>2.73</v>
+        <v>3.05</v>
       </c>
       <c r="V61" s="3" t="n">
-        <v>3.52</v>
+        <v>3.61</v>
       </c>
       <c r="W61" s="3" t="n">
-        <v>3.88</v>
+        <v>3.83</v>
       </c>
       <c r="X61" s="3" t="n">
-        <v>3.12</v>
+        <v>3.18</v>
       </c>
       <c r="Y61" s="3" t="n">
-        <v>2.9</v>
+        <v>2.72</v>
       </c>
       <c r="Z61" s="3" t="n">
         <v>2.47</v>
@@ -5690,76 +5690,76 @@
         </is>
       </c>
       <c r="C64" s="3" t="n">
-        <v>50.06</v>
+        <v>47.73</v>
       </c>
       <c r="D64" s="3" t="n">
+        <v>43.45</v>
+      </c>
+      <c r="E64" s="3" t="n">
         <v>38.2</v>
       </c>
-      <c r="E64" s="3" t="n">
-        <v>37.87</v>
-      </c>
       <c r="F64" s="3" t="n">
-        <v>38.09</v>
+        <v>38.25</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>38.35</v>
+        <v>38.01</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>38.05</v>
+        <v>37.8</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>52.4</v>
+        <v>43.5</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>45.83</v>
+        <v>51.18</v>
       </c>
       <c r="K64" s="3" t="n">
+        <v>45.46</v>
+      </c>
+      <c r="L64" s="3" t="n">
+        <v>39.72</v>
+      </c>
+      <c r="M64" s="3" t="n">
+        <v>40.12</v>
+      </c>
+      <c r="N64" s="3" t="n">
+        <v>40.38</v>
+      </c>
+      <c r="O64" s="3" t="n">
+        <v>38.15</v>
+      </c>
+      <c r="P64" s="3" t="n">
         <v>40.29</v>
       </c>
-      <c r="L64" s="3" t="n">
-        <v>38.59</v>
-      </c>
-      <c r="M64" s="3" t="n">
-        <v>37.96</v>
-      </c>
-      <c r="N64" s="3" t="n">
-        <v>43.69</v>
-      </c>
-      <c r="O64" s="3" t="n">
-        <v>39.72</v>
-      </c>
-      <c r="P64" s="3" t="n">
-        <v>43.35</v>
-      </c>
       <c r="Q64" s="3" t="n">
-        <v>40.25</v>
+        <v>40.24</v>
       </c>
       <c r="R64" s="3" t="n">
-        <v>43.47</v>
+        <v>40.16</v>
       </c>
       <c r="S64" s="3" t="n">
-        <v>60.86</v>
+        <v>57.29</v>
       </c>
       <c r="T64" s="3" t="n">
-        <v>56.48</v>
+        <v>56.38</v>
       </c>
       <c r="U64" s="3" t="n">
-        <v>50.47</v>
+        <v>56.53</v>
       </c>
       <c r="V64" s="3" t="n">
-        <v>67.48999999999999</v>
+        <v>70.72</v>
       </c>
       <c r="W64" s="3" t="n">
-        <v>73.19</v>
+        <v>72.20999999999999</v>
       </c>
       <c r="X64" s="3" t="n">
-        <v>59.86</v>
+        <v>61.04</v>
       </c>
       <c r="Y64" s="3" t="n">
-        <v>55.65</v>
+        <v>53.09</v>
       </c>
       <c r="Z64" s="3" t="n">
-        <v>43.97</v>
+        <v>44.06</v>
       </c>
     </row>
     <row r="65">
@@ -5858,76 +5858,76 @@
         </is>
       </c>
       <c r="C66" s="3" t="n">
-        <v>3.25</v>
+        <v>3.1</v>
       </c>
       <c r="D66" s="3" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="E66" s="3" t="n">
         <v>2.52</v>
       </c>
-      <c r="E66" s="3" t="n">
+      <c r="F66" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="G66" s="3" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="H66" s="3" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="I66" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J66" s="3" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="K66" s="3" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="L66" s="3" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="M66" s="3" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="N66" s="3" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="O66" s="3" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="P66" s="3" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="Q66" s="3" t="n">
         <v>2.5</v>
       </c>
-      <c r="F66" s="3" t="n">
-        <v>2.55</v>
-      </c>
-      <c r="G66" s="3" t="n">
+      <c r="R66" s="3" t="n">
         <v>2.53</v>
       </c>
-      <c r="H66" s="3" t="n">
-        <v>2.47</v>
-      </c>
-      <c r="I66" s="3" t="n">
-        <v>3.62</v>
-      </c>
-      <c r="J66" s="3" t="n">
-        <v>3.07</v>
-      </c>
-      <c r="K66" s="3" t="n">
-        <v>2.58</v>
-      </c>
-      <c r="L66" s="3" t="n">
-        <v>2.35</v>
-      </c>
-      <c r="M66" s="3" t="n">
-        <v>2.28</v>
-      </c>
-      <c r="N66" s="3" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="O66" s="3" t="n">
-        <v>2.38</v>
-      </c>
-      <c r="P66" s="3" t="n">
-        <v>2.73</v>
-      </c>
-      <c r="Q66" s="3" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="R66" s="3" t="n">
-        <v>2.74</v>
-      </c>
       <c r="S66" s="3" t="n">
-        <v>4.32</v>
+        <v>4.12</v>
       </c>
       <c r="T66" s="3" t="n">
         <v>4.12</v>
       </c>
       <c r="U66" s="3" t="n">
-        <v>3.63</v>
+        <v>4.07</v>
       </c>
       <c r="V66" s="3" t="n">
-        <v>4.66</v>
+        <v>4.88</v>
       </c>
       <c r="W66" s="3" t="n">
-        <v>5.2</v>
+        <v>5.13</v>
       </c>
       <c r="X66" s="3" t="n">
-        <v>4.13</v>
+        <v>4.21</v>
       </c>
       <c r="Y66" s="3" t="n">
-        <v>3.78</v>
+        <v>3.56</v>
       </c>
       <c r="Z66" s="3" t="n">
-        <v>3.12</v>
+        <v>3.13</v>
       </c>
     </row>
     <row r="67">
@@ -6110,76 +6110,76 @@
         </is>
       </c>
       <c r="C69" s="3" t="n">
-        <v>50.6</v>
+        <v>48.3</v>
       </c>
       <c r="D69" s="3" t="n">
+        <v>43.92</v>
+      </c>
+      <c r="E69" s="3" t="n">
         <v>38.66</v>
       </c>
-      <c r="E69" s="3" t="n">
-        <v>38.33</v>
-      </c>
       <c r="F69" s="3" t="n">
-        <v>38.55</v>
+        <v>38.66</v>
       </c>
       <c r="G69" s="3" t="n">
-        <v>38.81</v>
+        <v>38.42</v>
       </c>
       <c r="H69" s="3" t="n">
-        <v>38.46</v>
+        <v>38.21</v>
       </c>
       <c r="I69" s="3" t="n">
-        <v>52.97</v>
+        <v>43.97</v>
       </c>
       <c r="J69" s="3" t="n">
-        <v>46.27</v>
+        <v>51.67</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>40.77</v>
+        <v>46</v>
       </c>
       <c r="L69" s="3" t="n">
-        <v>39.01</v>
+        <v>40.15</v>
       </c>
       <c r="M69" s="3" t="n">
-        <v>38.37</v>
+        <v>40.59</v>
       </c>
       <c r="N69" s="3" t="n">
-        <v>44.21</v>
+        <v>40.86</v>
       </c>
       <c r="O69" s="3" t="n">
-        <v>40.19</v>
+        <v>38.6</v>
       </c>
       <c r="P69" s="3" t="n">
-        <v>43.91</v>
+        <v>40.81</v>
       </c>
       <c r="Q69" s="3" t="n">
-        <v>40.68</v>
+        <v>40.72</v>
       </c>
       <c r="R69" s="3" t="n">
-        <v>43.94</v>
+        <v>40.59</v>
       </c>
       <c r="S69" s="3" t="n">
-        <v>61.52</v>
+        <v>57.85</v>
       </c>
       <c r="T69" s="3" t="n">
-        <v>56.97</v>
+        <v>56.93</v>
       </c>
       <c r="U69" s="3" t="n">
-        <v>50.91</v>
+        <v>57.02</v>
       </c>
       <c r="V69" s="3" t="n">
-        <v>68.15000000000001</v>
+        <v>71.34</v>
       </c>
       <c r="W69" s="3" t="n">
-        <v>73.90000000000001</v>
+        <v>72.83</v>
       </c>
       <c r="X69" s="3" t="n">
-        <v>60.44</v>
+        <v>61.63</v>
       </c>
       <c r="Y69" s="3" t="n">
-        <v>56.19</v>
+        <v>53.61</v>
       </c>
       <c r="Z69" s="3" t="n">
-        <v>44.45</v>
+        <v>44.54</v>
       </c>
     </row>
     <row r="70">
@@ -6278,76 +6278,76 @@
         </is>
       </c>
       <c r="C71" s="3" t="n">
-        <v>3.79</v>
+        <v>3.67</v>
       </c>
       <c r="D71" s="3" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="E71" s="3" t="n">
         <v>2.98</v>
       </c>
-      <c r="E71" s="3" t="n">
-        <v>2.95</v>
-      </c>
       <c r="F71" s="3" t="n">
-        <v>3.01</v>
+        <v>3.02</v>
       </c>
       <c r="G71" s="3" t="n">
-        <v>2.99</v>
+        <v>2.88</v>
       </c>
       <c r="H71" s="3" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="I71" s="3" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="J71" s="3" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="K71" s="3" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="L71" s="3" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="M71" s="3" t="n">
         <v>2.88</v>
       </c>
-      <c r="I71" s="3" t="n">
-        <v>4.18</v>
-      </c>
-      <c r="J71" s="3" t="n">
-        <v>3.52</v>
-      </c>
-      <c r="K71" s="3" t="n">
+      <c r="N71" s="3" t="n">
         <v>3.06</v>
       </c>
-      <c r="L71" s="3" t="n">
-        <v>2.77</v>
-      </c>
-      <c r="M71" s="3" t="n">
-        <v>2.69</v>
-      </c>
-      <c r="N71" s="3" t="n">
-        <v>3.32</v>
-      </c>
       <c r="O71" s="3" t="n">
-        <v>2.85</v>
+        <v>2.74</v>
       </c>
       <c r="P71" s="3" t="n">
-        <v>3.29</v>
+        <v>3.06</v>
       </c>
       <c r="Q71" s="3" t="n">
         <v>2.97</v>
       </c>
       <c r="R71" s="3" t="n">
-        <v>3.21</v>
+        <v>2.96</v>
       </c>
       <c r="S71" s="3" t="n">
-        <v>4.98</v>
+        <v>4.69</v>
       </c>
       <c r="T71" s="3" t="n">
-        <v>4.61</v>
+        <v>4.67</v>
       </c>
       <c r="U71" s="3" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="V71" s="3" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="W71" s="3" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="X71" s="3" t="n">
+        <v>4.81</v>
+      </c>
+      <c r="Y71" s="3" t="n">
         <v>4.07</v>
       </c>
-      <c r="V71" s="3" t="n">
-        <v>5.32</v>
-      </c>
-      <c r="W71" s="3" t="n">
-        <v>5.91</v>
-      </c>
-      <c r="X71" s="3" t="n">
-        <v>4.71</v>
-      </c>
-      <c r="Y71" s="3" t="n">
-        <v>4.33</v>
-      </c>
       <c r="Z71" s="3" t="n">
-        <v>3.6</v>
+        <v>3.61</v>
       </c>
     </row>
     <row r="72">
@@ -6530,76 +6530,76 @@
         </is>
       </c>
       <c r="C74" s="3" t="n">
-        <v>48.8</v>
+        <v>46.54</v>
       </c>
       <c r="D74" s="3" t="n">
-        <v>37.29</v>
+        <v>42.49</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>37.08</v>
+        <v>37.4</v>
       </c>
       <c r="F74" s="3" t="n">
-        <v>37.26</v>
+        <v>37.37</v>
       </c>
       <c r="G74" s="3" t="n">
-        <v>37.39</v>
+        <v>37.02</v>
       </c>
       <c r="H74" s="3" t="n">
-        <v>37.06</v>
+        <v>36.81</v>
       </c>
       <c r="I74" s="3" t="n">
-        <v>50.87</v>
+        <v>42.23</v>
       </c>
       <c r="J74" s="3" t="n">
-        <v>44.63</v>
+        <v>49.69</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>39.12</v>
+        <v>44.18</v>
       </c>
       <c r="L74" s="3" t="n">
-        <v>37.63</v>
+        <v>38.69</v>
       </c>
       <c r="M74" s="3" t="n">
-        <v>37.17</v>
+        <v>39.32</v>
       </c>
       <c r="N74" s="3" t="n">
-        <v>42.77</v>
+        <v>39.54</v>
       </c>
       <c r="O74" s="3" t="n">
-        <v>38.81</v>
+        <v>37.27</v>
       </c>
       <c r="P74" s="3" t="n">
-        <v>42.31</v>
+        <v>39.32</v>
       </c>
       <c r="Q74" s="3" t="n">
-        <v>39.37</v>
+        <v>39.4</v>
       </c>
       <c r="R74" s="3" t="n">
-        <v>42.43</v>
+        <v>39.2</v>
       </c>
       <c r="S74" s="3" t="n">
-        <v>59.27</v>
+        <v>55.79</v>
       </c>
       <c r="T74" s="3" t="n">
-        <v>54.88</v>
+        <v>54.78</v>
       </c>
       <c r="U74" s="3" t="n">
-        <v>48.99</v>
+        <v>54.87</v>
       </c>
       <c r="V74" s="3" t="n">
-        <v>65.59</v>
+        <v>68.66</v>
       </c>
       <c r="W74" s="3" t="n">
-        <v>71.34</v>
+        <v>70.31999999999999</v>
       </c>
       <c r="X74" s="3" t="n">
-        <v>58.29</v>
+        <v>59.44</v>
       </c>
       <c r="Y74" s="3" t="n">
-        <v>54.42</v>
+        <v>51.92</v>
       </c>
       <c r="Z74" s="3" t="n">
-        <v>43</v>
+        <v>43.09</v>
       </c>
     </row>
     <row r="75">
@@ -6698,73 +6698,73 @@
         </is>
       </c>
       <c r="C76" s="3" t="n">
-        <v>2</v>
+        <v>1.91</v>
       </c>
       <c r="D76" s="3" t="n">
-        <v>1.6</v>
+        <v>1.91</v>
       </c>
       <c r="E76" s="3" t="n">
-        <v>1.71</v>
+        <v>1.72</v>
       </c>
       <c r="F76" s="3" t="n">
-        <v>1.71</v>
+        <v>1.72</v>
       </c>
       <c r="G76" s="3" t="n">
-        <v>1.57</v>
+        <v>1.48</v>
       </c>
       <c r="H76" s="3" t="n">
-        <v>1.48</v>
+        <v>1.47</v>
       </c>
       <c r="I76" s="3" t="n">
-        <v>2.09</v>
+        <v>1.73</v>
       </c>
       <c r="J76" s="3" t="n">
-        <v>1.87</v>
+        <v>1.89</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>1.41</v>
+        <v>1.63</v>
       </c>
       <c r="L76" s="3" t="n">
         <v>1.39</v>
       </c>
       <c r="M76" s="3" t="n">
-        <v>1.49</v>
+        <v>1.61</v>
       </c>
       <c r="N76" s="3" t="n">
-        <v>1.88</v>
+        <v>1.74</v>
       </c>
       <c r="O76" s="3" t="n">
-        <v>1.47</v>
+        <v>1.42</v>
       </c>
       <c r="P76" s="3" t="n">
-        <v>1.69</v>
+        <v>1.57</v>
       </c>
       <c r="Q76" s="3" t="n">
         <v>1.65</v>
       </c>
       <c r="R76" s="3" t="n">
-        <v>1.7</v>
+        <v>1.57</v>
       </c>
       <c r="S76" s="3" t="n">
-        <v>2.73</v>
+        <v>2.62</v>
       </c>
       <c r="T76" s="3" t="n">
         <v>2.52</v>
       </c>
       <c r="U76" s="3" t="n">
-        <v>2.16</v>
+        <v>2.41</v>
       </c>
       <c r="V76" s="3" t="n">
-        <v>2.75</v>
+        <v>2.82</v>
       </c>
       <c r="W76" s="3" t="n">
-        <v>3.35</v>
+        <v>3.23</v>
       </c>
       <c r="X76" s="3" t="n">
-        <v>2.56</v>
+        <v>2.62</v>
       </c>
       <c r="Y76" s="3" t="n">
-        <v>2.56</v>
+        <v>2.39</v>
       </c>
       <c r="Z76" s="3" t="n">
         <v>2.15</v>
@@ -6950,76 +6950,76 @@
         </is>
       </c>
       <c r="C79" s="3" t="n">
-        <v>46.8</v>
+        <v>44.63</v>
       </c>
       <c r="D79" s="3" t="n">
+        <v>40.58</v>
+      </c>
+      <c r="E79" s="3" t="n">
         <v>35.68</v>
       </c>
-      <c r="E79" s="3" t="n">
-        <v>35.38</v>
-      </c>
       <c r="F79" s="3" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="G79" s="3" t="n">
         <v>35.54</v>
       </c>
-      <c r="G79" s="3" t="n">
-        <v>35.82</v>
-      </c>
       <c r="H79" s="3" t="n">
-        <v>35.58</v>
+        <v>35.34</v>
       </c>
       <c r="I79" s="3" t="n">
-        <v>48.78</v>
+        <v>40.5</v>
       </c>
       <c r="J79" s="3" t="n">
-        <v>42.76</v>
+        <v>47.8</v>
       </c>
       <c r="K79" s="3" t="n">
+        <v>42.55</v>
+      </c>
+      <c r="L79" s="3" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="M79" s="3" t="n">
         <v>37.71</v>
       </c>
-      <c r="L79" s="3" t="n">
-        <v>36.24</v>
-      </c>
-      <c r="M79" s="3" t="n">
-        <v>35.68</v>
-      </c>
       <c r="N79" s="3" t="n">
-        <v>40.89</v>
+        <v>37.8</v>
       </c>
       <c r="O79" s="3" t="n">
-        <v>37.33</v>
+        <v>35.86</v>
       </c>
       <c r="P79" s="3" t="n">
-        <v>40.62</v>
+        <v>37.75</v>
       </c>
       <c r="Q79" s="3" t="n">
-        <v>37.71</v>
+        <v>37.75</v>
       </c>
       <c r="R79" s="3" t="n">
-        <v>40.74</v>
+        <v>37.63</v>
       </c>
       <c r="S79" s="3" t="n">
-        <v>56.54</v>
+        <v>53.16</v>
       </c>
       <c r="T79" s="3" t="n">
-        <v>52.35</v>
+        <v>52.26</v>
       </c>
       <c r="U79" s="3" t="n">
-        <v>46.84</v>
+        <v>52.46</v>
       </c>
       <c r="V79" s="3" t="n">
-        <v>62.83</v>
+        <v>65.84</v>
       </c>
       <c r="W79" s="3" t="n">
-        <v>67.98999999999999</v>
+        <v>67.08</v>
       </c>
       <c r="X79" s="3" t="n">
-        <v>55.73</v>
+        <v>56.83</v>
       </c>
       <c r="Y79" s="3" t="n">
-        <v>51.86</v>
+        <v>49.53</v>
       </c>
       <c r="Z79" s="3" t="n">
-        <v>40.85</v>
+        <v>40.93</v>
       </c>
     </row>
     <row r="80">
@@ -7370,76 +7370,76 @@
         </is>
       </c>
       <c r="C84" s="3" t="n">
-        <v>49.9</v>
+        <v>47.18</v>
       </c>
       <c r="D84" s="3" t="n">
-        <v>38.08</v>
+        <v>43.26</v>
       </c>
       <c r="E84" s="3" t="n">
-        <v>36.54</v>
+        <v>37.05</v>
       </c>
       <c r="F84" s="3" t="n">
-        <v>37.45</v>
+        <v>37.64</v>
       </c>
       <c r="G84" s="3" t="n">
-        <v>36.41</v>
+        <v>36.08</v>
       </c>
       <c r="H84" s="3" t="n">
-        <v>35.94</v>
+        <v>35.59</v>
       </c>
       <c r="I84" s="3" t="n">
-        <v>45.8</v>
+        <v>38.03</v>
       </c>
       <c r="J84" s="3" t="n">
-        <v>39.33</v>
+        <v>44.18</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>34.44</v>
+        <v>39.21</v>
       </c>
       <c r="L84" s="3" t="n">
-        <v>34.45</v>
+        <v>35.86</v>
       </c>
       <c r="M84" s="3" t="n">
-        <v>34.61</v>
+        <v>36.86</v>
       </c>
       <c r="N84" s="3" t="n">
-        <v>39.39</v>
+        <v>36.91</v>
       </c>
       <c r="O84" s="3" t="n">
-        <v>35.39</v>
+        <v>34.48</v>
       </c>
       <c r="P84" s="3" t="n">
-        <v>14.5</v>
+        <v>35.45</v>
       </c>
       <c r="Q84" s="3" t="n">
-        <v>12.9</v>
+        <v>35.68</v>
       </c>
       <c r="R84" s="3" t="n">
-        <v>12.75</v>
+        <v>35.6</v>
       </c>
       <c r="S84" s="3" t="n">
-        <v>52.99</v>
+        <v>49.97</v>
       </c>
       <c r="T84" s="3" t="n">
-        <v>49.39</v>
+        <v>49.44</v>
       </c>
       <c r="U84" s="3" t="n">
-        <v>17.31</v>
+        <v>46.05</v>
       </c>
       <c r="V84" s="3" t="n">
-        <v>59.84</v>
+        <v>62.71</v>
       </c>
       <c r="W84" s="3" t="n">
-        <v>64.81</v>
+        <v>23.55</v>
       </c>
       <c r="X84" s="3" t="n">
-        <v>53.18</v>
+        <v>54.33</v>
       </c>
       <c r="Y84" s="3" t="n">
-        <v>19.98</v>
+        <v>47.22</v>
       </c>
       <c r="Z84" s="3" t="n">
-        <v>39.13</v>
+        <v>39.17</v>
       </c>
     </row>
     <row r="85">
@@ -7493,13 +7493,13 @@
         <v>0</v>
       </c>
       <c r="P85" s="3" t="n">
-        <v>-23.21</v>
+        <v>0</v>
       </c>
       <c r="Q85" s="3" t="n">
-        <v>-22.28</v>
+        <v>0</v>
       </c>
       <c r="R85" s="3" t="n">
-        <v>-25.28</v>
+        <v>0</v>
       </c>
       <c r="S85" s="3" t="n">
         <v>0</v>
@@ -7508,19 +7508,19 @@
         <v>0</v>
       </c>
       <c r="U85" s="3" t="n">
-        <v>-23.85</v>
+        <v>0</v>
       </c>
       <c r="V85" s="3" t="n">
         <v>0</v>
       </c>
       <c r="W85" s="3" t="n">
-        <v>0</v>
+        <v>-40.21</v>
       </c>
       <c r="X85" s="3" t="n">
         <v>0</v>
       </c>
       <c r="Y85" s="3" t="n">
-        <v>-29.65</v>
+        <v>0</v>
       </c>
       <c r="Z85" s="3" t="n">
         <v>0</v>
@@ -7538,76 +7538,76 @@
         </is>
       </c>
       <c r="C86" s="3" t="n">
-        <v>3.09</v>
+        <v>2.55</v>
       </c>
       <c r="D86" s="3" t="n">
-        <v>2.4</v>
+        <v>2.68</v>
       </c>
       <c r="E86" s="3" t="n">
-        <v>1.17</v>
+        <v>1.37</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>1.91</v>
+        <v>2</v>
       </c>
       <c r="G86" s="3" t="n">
-        <v>0.58</v>
+        <v>0.54</v>
       </c>
       <c r="H86" s="3" t="n">
-        <v>0.36</v>
+        <v>0.25</v>
       </c>
       <c r="I86" s="3" t="n">
-        <v>-2.98</v>
+        <v>-2.47</v>
       </c>
       <c r="J86" s="3" t="n">
-        <v>-3.42</v>
+        <v>-3.62</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>-3.27</v>
+        <v>-3.33</v>
       </c>
       <c r="L86" s="3" t="n">
-        <v>-1.79</v>
+        <v>-1.43</v>
       </c>
       <c r="M86" s="3" t="n">
-        <v>-1.07</v>
+        <v>-0.85</v>
       </c>
       <c r="N86" s="3" t="n">
-        <v>-1.5</v>
+        <v>-0.89</v>
       </c>
       <c r="O86" s="3" t="n">
-        <v>-1.95</v>
+        <v>-1.38</v>
       </c>
       <c r="P86" s="3" t="n">
-        <v>-2.9</v>
+        <v>-2.3</v>
       </c>
       <c r="Q86" s="3" t="n">
-        <v>-2.53</v>
+        <v>-2.07</v>
       </c>
       <c r="R86" s="3" t="n">
-        <v>-2.7</v>
+        <v>-2.03</v>
       </c>
       <c r="S86" s="3" t="n">
-        <v>-3.55</v>
+        <v>-3.2</v>
       </c>
       <c r="T86" s="3" t="n">
-        <v>-2.96</v>
+        <v>-2.82</v>
       </c>
       <c r="U86" s="3" t="n">
-        <v>-5.68</v>
+        <v>-6.4</v>
       </c>
       <c r="V86" s="3" t="n">
-        <v>-2.99</v>
+        <v>-3.14</v>
       </c>
       <c r="W86" s="3" t="n">
-        <v>-3.18</v>
+        <v>-3.32</v>
       </c>
       <c r="X86" s="3" t="n">
-        <v>-2.55</v>
+        <v>-2.5</v>
       </c>
       <c r="Y86" s="3" t="n">
-        <v>-2.23</v>
+        <v>-2.31</v>
       </c>
       <c r="Z86" s="3" t="n">
-        <v>-1.72</v>
+        <v>-1.76</v>
       </c>
     </row>
     <row r="87">
@@ -7790,76 +7790,76 @@
         </is>
       </c>
       <c r="C89" s="3" t="n">
-        <v>46.07</v>
+        <v>44.01</v>
       </c>
       <c r="D89" s="3" t="n">
-        <v>34.78</v>
+        <v>39.9</v>
       </c>
       <c r="E89" s="3" t="n">
-        <v>34.58</v>
+        <v>34.85</v>
       </c>
       <c r="F89" s="3" t="n">
+        <v>35.02</v>
+      </c>
+      <c r="G89" s="3" t="n">
         <v>34.91</v>
       </c>
-      <c r="G89" s="3" t="n">
-        <v>35.22</v>
-      </c>
       <c r="H89" s="3" t="n">
-        <v>34.91</v>
+        <v>34.61</v>
       </c>
       <c r="I89" s="3" t="n">
-        <v>47.64</v>
+        <v>39.67</v>
       </c>
       <c r="J89" s="3" t="n">
-        <v>41.51</v>
+        <v>46.45</v>
       </c>
       <c r="K89" s="3" t="n">
+        <v>41.15</v>
+      </c>
+      <c r="L89" s="3" t="n">
+        <v>36.14</v>
+      </c>
+      <c r="M89" s="3" t="n">
         <v>36.61</v>
       </c>
-      <c r="L89" s="3" t="n">
-        <v>35.15</v>
-      </c>
-      <c r="M89" s="3" t="n">
-        <v>34.48</v>
-      </c>
       <c r="N89" s="3" t="n">
-        <v>39.78</v>
+        <v>36.62</v>
       </c>
       <c r="O89" s="3" t="n">
-        <v>36.49</v>
+        <v>34.81</v>
       </c>
       <c r="P89" s="3" t="n">
-        <v>39.67</v>
+        <v>36.65</v>
       </c>
       <c r="Q89" s="3" t="n">
-        <v>36.83</v>
+        <v>36.65</v>
       </c>
       <c r="R89" s="3" t="n">
-        <v>39.7</v>
+        <v>36.39</v>
       </c>
       <c r="S89" s="3" t="n">
-        <v>54.11</v>
+        <v>50.54</v>
       </c>
       <c r="T89" s="3" t="n">
-        <v>49.86</v>
+        <v>49.54</v>
       </c>
       <c r="U89" s="3" t="n">
-        <v>44.27</v>
+        <v>49.58</v>
       </c>
       <c r="V89" s="3" t="n">
-        <v>59.11</v>
+        <v>61.88</v>
       </c>
       <c r="W89" s="3" t="n">
-        <v>64.14</v>
+        <v>63.28</v>
       </c>
       <c r="X89" s="3" t="n">
-        <v>53.02</v>
+        <v>54.12</v>
       </c>
       <c r="Y89" s="3" t="n">
-        <v>49.96</v>
+        <v>47.86</v>
       </c>
       <c r="Z89" s="3" t="n">
-        <v>39.82</v>
+        <v>39.85</v>
       </c>
     </row>
     <row r="90">
@@ -7958,76 +7958,76 @@
         </is>
       </c>
       <c r="C91" s="3" t="n">
-        <v>-0.74</v>
+        <v>-0.62</v>
       </c>
       <c r="D91" s="3" t="n">
-        <v>-0.9</v>
+        <v>-0.68</v>
       </c>
       <c r="E91" s="3" t="n">
-        <v>-0.8</v>
+        <v>-0.84</v>
       </c>
       <c r="F91" s="3" t="n">
         <v>-0.63</v>
       </c>
       <c r="G91" s="3" t="n">
-        <v>-0.6</v>
+        <v>-0.63</v>
       </c>
       <c r="H91" s="3" t="n">
-        <v>-0.66</v>
+        <v>-0.73</v>
       </c>
       <c r="I91" s="3" t="n">
-        <v>-1.14</v>
+        <v>-0.83</v>
       </c>
       <c r="J91" s="3" t="n">
-        <v>-1.25</v>
+        <v>-1.35</v>
       </c>
       <c r="K91" s="3" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="L91" s="3" t="n">
+        <v>-1.16</v>
+      </c>
+      <c r="M91" s="3" t="n">
         <v>-1.1</v>
       </c>
-      <c r="L91" s="3" t="n">
-        <v>-1.09</v>
-      </c>
-      <c r="M91" s="3" t="n">
-        <v>-1.21</v>
-      </c>
       <c r="N91" s="3" t="n">
-        <v>-1.11</v>
+        <v>-1.17</v>
       </c>
       <c r="O91" s="3" t="n">
-        <v>-0.84</v>
+        <v>-1.04</v>
       </c>
       <c r="P91" s="3" t="n">
-        <v>-0.95</v>
+        <v>-1.1</v>
       </c>
       <c r="Q91" s="3" t="n">
-        <v>-0.88</v>
+        <v>-1.1</v>
       </c>
       <c r="R91" s="3" t="n">
-        <v>-1.03</v>
+        <v>-1.24</v>
       </c>
       <c r="S91" s="3" t="n">
-        <v>-2.43</v>
+        <v>-2.63</v>
       </c>
       <c r="T91" s="3" t="n">
-        <v>-2.49</v>
+        <v>-2.72</v>
       </c>
       <c r="U91" s="3" t="n">
-        <v>-2.57</v>
+        <v>-2.88</v>
       </c>
       <c r="V91" s="3" t="n">
-        <v>-3.72</v>
+        <v>-3.96</v>
       </c>
       <c r="W91" s="3" t="n">
-        <v>-3.85</v>
+        <v>-3.8</v>
       </c>
       <c r="X91" s="3" t="n">
-        <v>-2.7</v>
+        <v>-2.71</v>
       </c>
       <c r="Y91" s="3" t="n">
-        <v>-1.9</v>
+        <v>-1.68</v>
       </c>
       <c r="Z91" s="3" t="n">
-        <v>-1.04</v>
+        <v>-1.08</v>
       </c>
     </row>
     <row r="92">

</xml_diff>